<commit_message>
Small corrections to CellCount script and CellCount xlsx data file
</commit_message>
<xml_diff>
--- a/StatisticalAnalyses/Raji/data/data_counts_cleaned.xlsx
+++ b/StatisticalAnalyses/Raji/data/data_counts_cleaned.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Leander/Documents/Statistical_Analyses/2026/NeleF_Raji/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{446E95DD-D33B-E345-B19A-BC9B894C5F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B295EAE-B077-D545-830C-B5D8782BFF61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="560" yWindow="-20980" windowWidth="33720" windowHeight="20980" xr2:uid="{47F8F176-BF44-4A4C-9CFE-0EC8B11B1CF1}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17400" xr2:uid="{47F8F176-BF44-4A4C-9CFE-0EC8B11B1CF1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$242</definedName>
+  </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="27">
   <si>
     <t>Experiment</t>
   </si>
@@ -1013,7 +1016,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28924032-712C-42DD-811A-811BE3665EE3}">
-  <dimension ref="A1:G282"/>
+  <dimension ref="A1:G242"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
@@ -3997,7 +4000,7 @@
         <v>18</v>
       </c>
       <c r="B162">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C162">
         <v>1</v>
@@ -4006,7 +4009,7 @@
         <v>2</v>
       </c>
       <c r="E162" s="3">
-        <v>6.1058758878961186E-2</v>
+        <v>1.0577657636481166</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.2">
@@ -4014,7 +4017,7 @@
         <v>18</v>
       </c>
       <c r="B163">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C163">
         <v>2</v>
@@ -4023,7 +4026,7 @@
         <v>2</v>
       </c>
       <c r="E163" s="3">
-        <v>0.11962914963612802</v>
+        <v>0.17460640805517563</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.2">
@@ -4031,7 +4034,7 @@
         <v>18</v>
       </c>
       <c r="B164">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C164">
         <v>3</v>
@@ -4040,7 +4043,7 @@
         <v>19</v>
       </c>
       <c r="E164" s="3">
-        <v>9.3357699030669004</v>
+        <v>19.991828952744111</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.2">
@@ -4048,7 +4051,7 @@
         <v>18</v>
       </c>
       <c r="B165">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C165">
         <v>4</v>
@@ -4057,7 +4060,7 @@
         <v>19</v>
       </c>
       <c r="E165" s="3">
-        <v>12.504211006083665</v>
+        <v>2.6998689384010488</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.2">
@@ -4065,7 +4068,7 @@
         <v>18</v>
       </c>
       <c r="B166">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C166">
         <v>5</v>
@@ -4074,7 +4077,7 @@
         <v>20</v>
       </c>
       <c r="E166" s="3">
-        <v>7.0165208940719141</v>
+        <v>211.32042560613991</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.2">
@@ -4082,7 +4085,7 @@
         <v>18</v>
       </c>
       <c r="B167">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C167">
         <v>6</v>
@@ -4091,7 +4094,7 @@
         <v>20</v>
       </c>
       <c r="E167" s="3">
-        <v>6.2174046426014931</v>
+        <v>41.197975253093361</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.2">
@@ -4099,7 +4102,7 @@
         <v>18</v>
       </c>
       <c r="B168">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C168">
         <v>7</v>
@@ -4108,7 +4111,7 @@
         <v>2</v>
       </c>
       <c r="E168" s="3">
-        <v>2.1277501170262562E-2</v>
+        <v>0.12223071046600459</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.2">
@@ -4116,7 +4119,7 @@
         <v>18</v>
       </c>
       <c r="B169">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C169">
         <v>8</v>
@@ -4125,7 +4128,7 @@
         <v>2</v>
       </c>
       <c r="E169" s="3">
-        <v>7.8514505554901276E-2</v>
+        <v>0.52889433247967932</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.2">
@@ -4133,7 +4136,7 @@
         <v>18</v>
       </c>
       <c r="B170">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C170">
         <v>9</v>
@@ -4142,7 +4145,7 @@
         <v>19</v>
       </c>
       <c r="E170" s="3">
-        <v>12.947715109098393</v>
+        <v>3.4331895242146198</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.2">
@@ -4150,7 +4153,7 @@
         <v>18</v>
       </c>
       <c r="B171">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C171">
         <v>10</v>
@@ -4159,7 +4162,7 @@
         <v>19</v>
       </c>
       <c r="E171" s="3">
-        <v>12.576115842557909</v>
+        <v>5.0114458949452452</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.2">
@@ -4167,7 +4170,7 @@
         <v>18</v>
       </c>
       <c r="B172">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C172">
         <v>11</v>
@@ -4176,7 +4179,7 @@
         <v>20</v>
       </c>
       <c r="E172" s="3">
-        <v>5.3667656439019025</v>
+        <v>43.878424657534246</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.2">
@@ -4184,7 +4187,7 @@
         <v>18</v>
       </c>
       <c r="B173">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C173">
         <v>12</v>
@@ -4193,7 +4196,7 @@
         <v>20</v>
       </c>
       <c r="E173" s="3">
-        <v>5.0911448402105099</v>
+        <v>47.487810048759798</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.2">
@@ -4201,7 +4204,7 @@
         <v>18</v>
       </c>
       <c r="B174">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C174">
         <v>14</v>
@@ -4210,7 +4213,7 @@
         <v>19</v>
       </c>
       <c r="E174" s="3">
-        <v>11.629973343864153</v>
+        <v>9.0045298862004195</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.2">
@@ -4218,7 +4221,7 @@
         <v>18</v>
       </c>
       <c r="B175">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C175">
         <v>15</v>
@@ -4227,7 +4230,7 @@
         <v>20</v>
       </c>
       <c r="E175" s="3">
-        <v>9.7124145151589403</v>
+        <v>20.851735860167562</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.2">
@@ -4235,7 +4238,7 @@
         <v>18</v>
       </c>
       <c r="B176">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C176">
         <v>16</v>
@@ -4244,15 +4247,15 @@
         <v>2</v>
       </c>
       <c r="E176" s="3">
-        <v>0.10066033177645353</v>
-      </c>
-    </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
+        <v>0.36572328813368588</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>18</v>
       </c>
       <c r="B177">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C177">
         <v>17</v>
@@ -4261,15 +4264,15 @@
         <v>2</v>
       </c>
       <c r="E177" s="3">
-        <v>3.9688051911971896E-2</v>
-      </c>
-    </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
+        <v>0.61462814996926873</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>18</v>
       </c>
       <c r="B178">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C178">
         <v>18</v>
@@ -4278,15 +4281,15 @@
         <v>19</v>
       </c>
       <c r="E178" s="3">
-        <v>6.5545511034496586</v>
-      </c>
-    </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
+        <v>17.784426161389511</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>18</v>
       </c>
       <c r="B179">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C179">
         <v>19</v>
@@ -4295,15 +4298,15 @@
         <v>20</v>
       </c>
       <c r="E179" s="3">
-        <v>9.3667157584683363</v>
-      </c>
-    </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
+        <v>21.577227635336023</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>18</v>
       </c>
       <c r="B180">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C180">
         <v>20</v>
@@ -4312,15 +4315,15 @@
         <v>2</v>
       </c>
       <c r="E180" s="3">
-        <v>0.65036684754994611</v>
-      </c>
-    </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
+        <v>0.25822741227440965</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>18</v>
       </c>
       <c r="B181">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C181">
         <v>21</v>
@@ -4329,15 +4332,15 @@
         <v>2</v>
       </c>
       <c r="E181" s="3">
-        <v>0.20123873622073651</v>
-      </c>
-    </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
+        <v>0.77259850630955451</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>18</v>
       </c>
       <c r="B182">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C182">
         <v>22</v>
@@ -4346,15 +4349,15 @@
         <v>19</v>
       </c>
       <c r="E182" s="3">
-        <v>6.8233980522300106</v>
-      </c>
-    </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
+        <v>4.7538082515007467</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>18</v>
       </c>
       <c r="B183">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C183">
         <v>23</v>
@@ -4363,15 +4366,15 @@
         <v>19</v>
       </c>
       <c r="E183" s="3">
-        <v>5.2507945281193864</v>
-      </c>
-    </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
+        <v>5.8993923979087182</v>
+      </c>
+    </row>
+    <row r="184" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>18</v>
       </c>
       <c r="B184">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C184">
         <v>24</v>
@@ -4380,15 +4383,15 @@
         <v>20</v>
       </c>
       <c r="E184" s="3">
-        <v>6.7553056482945779</v>
-      </c>
-    </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
+        <v>117.60964548420995</v>
+      </c>
+    </row>
+    <row r="185" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>18</v>
       </c>
       <c r="B185">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C185">
         <v>25</v>
@@ -4397,984 +4400,1101 @@
         <v>20</v>
       </c>
       <c r="E185" s="3">
-        <v>3.5118144374593543</v>
-      </c>
-    </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
+        <v>31.239992883828506</v>
+      </c>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B186">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C186">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D186" t="s">
         <v>2</v>
       </c>
       <c r="E186" s="3">
-        <v>1.0577657636481166</v>
-      </c>
-    </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
+        <v>0.2763957987838585</v>
+      </c>
+      <c r="F186">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
+        <v>21</v>
+      </c>
+      <c r="B187">
+        <v>21</v>
+      </c>
+      <c r="C187">
+        <v>3</v>
+      </c>
+      <c r="D187" t="s">
+        <v>19</v>
+      </c>
+      <c r="E187" s="3">
+        <v>6.1667488899851994</v>
+      </c>
+      <c r="F187">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A188" t="s">
+        <v>21</v>
+      </c>
+      <c r="B188">
+        <v>21</v>
+      </c>
+      <c r="C188">
+        <v>4</v>
+      </c>
+      <c r="D188" t="s">
+        <v>2</v>
+      </c>
+      <c r="E188" s="3">
+        <v>0.18428424001179419</v>
+      </c>
+      <c r="F188">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A189" t="s">
+        <v>21</v>
+      </c>
+      <c r="B189">
+        <v>21</v>
+      </c>
+      <c r="C189">
+        <v>5</v>
+      </c>
+      <c r="D189" t="s">
+        <v>19</v>
+      </c>
+      <c r="E189" s="3">
+        <v>6.6952914635033842</v>
+      </c>
+      <c r="F189">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A190" t="s">
+        <v>21</v>
+      </c>
+      <c r="B190">
+        <v>21</v>
+      </c>
+      <c r="C190">
+        <v>6</v>
+      </c>
+      <c r="D190" t="s">
+        <v>20</v>
+      </c>
+      <c r="F190">
+        <v>1</v>
+      </c>
+      <c r="G190" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A191" t="s">
+        <v>21</v>
+      </c>
+      <c r="B191">
+        <v>21</v>
+      </c>
+      <c r="C191">
+        <v>7</v>
+      </c>
+      <c r="D191" t="s">
+        <v>2</v>
+      </c>
+      <c r="E191" s="3">
+        <v>0.74211502782931349</v>
+      </c>
+      <c r="F191">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A192" t="s">
+        <v>21</v>
+      </c>
+      <c r="B192">
+        <v>21</v>
+      </c>
+      <c r="C192">
+        <v>9</v>
+      </c>
+      <c r="D192" t="s">
+        <v>19</v>
+      </c>
+      <c r="E192" s="3">
+        <v>15.261446084563422</v>
+      </c>
+      <c r="F192">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="193" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A193" t="s">
+        <v>21</v>
+      </c>
+      <c r="B193">
+        <v>21</v>
+      </c>
+      <c r="C193">
+        <v>10</v>
+      </c>
+      <c r="D193" t="s">
+        <v>19</v>
+      </c>
+      <c r="F193">
+        <v>1</v>
+      </c>
+      <c r="G193" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="194" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A194" t="s">
+        <v>21</v>
+      </c>
+      <c r="B194">
+        <v>21</v>
+      </c>
+      <c r="C194">
+        <v>11</v>
+      </c>
+      <c r="D194" t="s">
+        <v>20</v>
+      </c>
+      <c r="E194" s="3">
+        <v>104.56226880394576</v>
+      </c>
+      <c r="F194">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A195" t="s">
+        <v>21</v>
+      </c>
+      <c r="B195">
+        <v>21</v>
+      </c>
+      <c r="C195">
+        <v>12</v>
+      </c>
+      <c r="D195" t="s">
+        <v>20</v>
+      </c>
+      <c r="F195">
+        <v>1</v>
+      </c>
+      <c r="G195" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A196" t="s">
+        <v>21</v>
+      </c>
+      <c r="B196">
+        <v>21</v>
+      </c>
+      <c r="C196">
+        <v>13</v>
+      </c>
+      <c r="D196" t="s">
+        <v>2</v>
+      </c>
+      <c r="E196" s="3">
+        <v>1.0822510822510825</v>
+      </c>
+      <c r="F196">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A197" t="s">
+        <v>21</v>
+      </c>
+      <c r="B197">
+        <v>21</v>
+      </c>
+      <c r="C197">
+        <v>14</v>
+      </c>
+      <c r="D197" t="s">
+        <v>20</v>
+      </c>
+      <c r="E197" s="3">
+        <v>31.99327498392919</v>
+      </c>
+      <c r="F197">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A198" t="s">
+        <v>21</v>
+      </c>
+      <c r="B198">
+        <v>21</v>
+      </c>
+      <c r="C198">
+        <v>15</v>
+      </c>
+      <c r="D198" t="s">
+        <v>2</v>
+      </c>
+      <c r="E198" s="3">
+        <v>4.4904661371937928</v>
+      </c>
+      <c r="F198">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A199" t="s">
+        <v>21</v>
+      </c>
+      <c r="B199">
+        <v>21</v>
+      </c>
+      <c r="C199">
+        <v>16</v>
+      </c>
+      <c r="D199" t="s">
+        <v>19</v>
+      </c>
+      <c r="E199" s="3">
+        <v>10.916747651441529</v>
+      </c>
+      <c r="F199">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A200" t="s">
+        <v>21</v>
+      </c>
+      <c r="B200">
+        <v>21</v>
+      </c>
+      <c r="C200">
+        <v>17</v>
+      </c>
+      <c r="D200" t="s">
+        <v>19</v>
+      </c>
+      <c r="E200" s="3">
+        <v>35.679978043090436</v>
+      </c>
+      <c r="F200">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A201" t="s">
+        <v>21</v>
+      </c>
+      <c r="B201">
+        <v>21</v>
+      </c>
+      <c r="C201">
         <v>18</v>
       </c>
-      <c r="B187">
-        <v>20</v>
-      </c>
-      <c r="C187">
+      <c r="D201" t="s">
+        <v>20</v>
+      </c>
+      <c r="E201" s="3">
+        <v>198.10997218305835</v>
+      </c>
+      <c r="F201">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A202" t="s">
+        <v>21</v>
+      </c>
+      <c r="B202">
+        <v>21</v>
+      </c>
+      <c r="C202">
+        <v>19</v>
+      </c>
+      <c r="D202" t="s">
+        <v>20</v>
+      </c>
+      <c r="E202" s="3">
+        <v>120.27829739752552</v>
+      </c>
+      <c r="F202">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="203" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A203" t="s">
+        <v>21</v>
+      </c>
+      <c r="B203">
+        <v>21</v>
+      </c>
+      <c r="C203">
+        <v>20</v>
+      </c>
+      <c r="D203" t="s">
         <v>2</v>
       </c>
-      <c r="D187" t="s">
-        <v>2</v>
-      </c>
-      <c r="E187" s="3">
-        <v>0.17460640805517563</v>
-      </c>
-    </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A188" t="s">
-        <v>18</v>
-      </c>
-      <c r="B188">
-        <v>20</v>
-      </c>
-      <c r="C188">
-        <v>3</v>
-      </c>
-      <c r="D188" t="s">
-        <v>19</v>
-      </c>
-      <c r="E188" s="3">
-        <v>19.991828952744111</v>
-      </c>
-    </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A189" t="s">
-        <v>18</v>
-      </c>
-      <c r="B189">
-        <v>20</v>
-      </c>
-      <c r="C189">
-        <v>4</v>
-      </c>
-      <c r="D189" t="s">
-        <v>19</v>
-      </c>
-      <c r="E189" s="3">
-        <v>2.6998689384010488</v>
-      </c>
-    </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A190" t="s">
-        <v>18</v>
-      </c>
-      <c r="B190">
-        <v>20</v>
-      </c>
-      <c r="C190">
-        <v>5</v>
-      </c>
-      <c r="D190" t="s">
-        <v>20</v>
-      </c>
-      <c r="E190" s="3">
-        <v>211.32042560613991</v>
-      </c>
-    </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A191" t="s">
-        <v>18</v>
-      </c>
-      <c r="B191">
-        <v>20</v>
-      </c>
-      <c r="C191">
+      <c r="E203" s="3">
+        <v>0.42121634319411594</v>
+      </c>
+      <c r="F203">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="204" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A204" t="s">
+        <v>21</v>
+      </c>
+      <c r="B204">
+        <v>21</v>
+      </c>
+      <c r="C204">
+        <v>21</v>
+      </c>
+      <c r="D204" t="s">
+        <v>19</v>
+      </c>
+      <c r="E204" s="3">
+        <v>21.348717447280077</v>
+      </c>
+      <c r="F204">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="205" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A205" t="s">
+        <v>21</v>
+      </c>
+      <c r="B205">
+        <v>21</v>
+      </c>
+      <c r="C205">
+        <v>22</v>
+      </c>
+      <c r="D205" t="s">
+        <v>19</v>
+      </c>
+      <c r="E205" s="3">
+        <v>7.5543545019039424</v>
+      </c>
+      <c r="F205">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="206" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A206" t="s">
+        <v>21</v>
+      </c>
+      <c r="B206">
+        <v>21</v>
+      </c>
+      <c r="C206">
+        <v>23</v>
+      </c>
+      <c r="D206" t="s">
+        <v>20</v>
+      </c>
+      <c r="E206" s="3">
+        <v>98.704866562009414</v>
+      </c>
+      <c r="F206">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="207" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A207" t="s">
+        <v>21</v>
+      </c>
+      <c r="B207">
+        <v>21</v>
+      </c>
+      <c r="C207">
+        <v>30</v>
+      </c>
+      <c r="D207" t="s">
+        <v>19</v>
+      </c>
+      <c r="E207" s="3">
+        <v>15.60758082497213</v>
+      </c>
+      <c r="F207">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="208" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A208" t="s">
+        <v>21</v>
+      </c>
+      <c r="B208">
+        <v>21</v>
+      </c>
+      <c r="C208">
+        <v>31</v>
+      </c>
+      <c r="D208" t="s">
+        <v>19</v>
+      </c>
+      <c r="E208" s="3">
+        <v>50.821000810494404</v>
+      </c>
+      <c r="F208">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A209" t="s">
+        <v>21</v>
+      </c>
+      <c r="B209">
+        <v>21</v>
+      </c>
+      <c r="C209">
+        <v>32</v>
+      </c>
+      <c r="D209" t="s">
+        <v>20</v>
+      </c>
+      <c r="E209" s="3">
+        <v>78.636660143509459</v>
+      </c>
+      <c r="F209">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A210" t="s">
+        <v>21</v>
+      </c>
+      <c r="B210">
+        <v>21</v>
+      </c>
+      <c r="C210">
+        <v>33</v>
+      </c>
+      <c r="D210" t="s">
+        <v>20</v>
+      </c>
+      <c r="E210" s="3">
+        <v>143.13526324699509</v>
+      </c>
+      <c r="F210">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A211" t="s">
+        <v>21</v>
+      </c>
+      <c r="B211">
+        <v>21</v>
+      </c>
+      <c r="C211">
+        <v>34</v>
+      </c>
+      <c r="D211" t="s">
+        <v>20</v>
+      </c>
+      <c r="E211" s="3">
+        <v>53.602376825947019</v>
+      </c>
+      <c r="F211">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A212" t="s">
+        <v>21</v>
+      </c>
+      <c r="B212">
+        <v>21</v>
+      </c>
+      <c r="C212">
+        <v>45</v>
+      </c>
+      <c r="D212" t="s">
+        <v>19</v>
+      </c>
+      <c r="E212" s="3">
+        <v>11.229837337507655</v>
+      </c>
+      <c r="F212">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A213" t="s">
+        <v>21</v>
+      </c>
+      <c r="B213">
+        <v>21</v>
+      </c>
+      <c r="C213">
+        <v>46</v>
+      </c>
+      <c r="D213" t="s">
+        <v>19</v>
+      </c>
+      <c r="E213" s="3">
+        <v>23.619957537154985</v>
+      </c>
+      <c r="F213">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A214" t="s">
+        <v>21</v>
+      </c>
+      <c r="B214">
+        <v>21</v>
+      </c>
+      <c r="C214">
+        <v>47</v>
+      </c>
+      <c r="D214" t="s">
+        <v>20</v>
+      </c>
+      <c r="E214" s="3">
+        <v>95.876870940412317</v>
+      </c>
+      <c r="F214">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A215" t="s">
+        <v>21</v>
+      </c>
+      <c r="B215">
+        <v>21</v>
+      </c>
+      <c r="C215">
+        <v>48</v>
+      </c>
+      <c r="D215" t="s">
+        <v>20</v>
+      </c>
+      <c r="E215" s="3">
+        <v>195.71214629147946</v>
+      </c>
+      <c r="F215">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="216" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A216" t="s">
+        <v>21</v>
+      </c>
+      <c r="B216">
+        <v>83</v>
+      </c>
+      <c r="C216">
         <v>6</v>
       </c>
-      <c r="D191" t="s">
-        <v>20</v>
-      </c>
-      <c r="E191" s="3">
-        <v>41.197975253093361</v>
-      </c>
-    </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A192" t="s">
-        <v>18</v>
-      </c>
-      <c r="B192">
-        <v>20</v>
-      </c>
-      <c r="C192">
-        <v>7</v>
-      </c>
-      <c r="D192" t="s">
-        <v>2</v>
-      </c>
-      <c r="E192" s="3">
-        <v>0.12223071046600459</v>
-      </c>
-    </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A193" t="s">
-        <v>18</v>
-      </c>
-      <c r="B193">
-        <v>20</v>
-      </c>
-      <c r="C193">
-        <v>8</v>
-      </c>
-      <c r="D193" t="s">
-        <v>2</v>
-      </c>
-      <c r="E193" s="3">
-        <v>0.52889433247967932</v>
-      </c>
-    </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A194" t="s">
-        <v>18</v>
-      </c>
-      <c r="B194">
-        <v>20</v>
-      </c>
-      <c r="C194">
-        <v>9</v>
-      </c>
-      <c r="D194" t="s">
-        <v>19</v>
-      </c>
-      <c r="E194" s="3">
-        <v>3.4331895242146198</v>
-      </c>
-    </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A195" t="s">
-        <v>18</v>
-      </c>
-      <c r="B195">
-        <v>20</v>
-      </c>
-      <c r="C195">
-        <v>10</v>
-      </c>
-      <c r="D195" t="s">
-        <v>19</v>
-      </c>
-      <c r="E195" s="3">
-        <v>5.0114458949452452</v>
-      </c>
-    </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A196" t="s">
-        <v>18</v>
-      </c>
-      <c r="B196">
-        <v>20</v>
-      </c>
-      <c r="C196">
+      <c r="D216" t="s">
+        <v>20</v>
+      </c>
+      <c r="E216" s="3">
+        <v>3.0286786384347364</v>
+      </c>
+      <c r="F216">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A217" t="s">
+        <v>21</v>
+      </c>
+      <c r="B217">
+        <v>83</v>
+      </c>
+      <c r="C217">
         <v>11</v>
       </c>
-      <c r="D196" t="s">
-        <v>20</v>
-      </c>
-      <c r="E196" s="3">
-        <v>43.878424657534246</v>
-      </c>
-    </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A197" t="s">
-        <v>18</v>
-      </c>
-      <c r="B197">
-        <v>20</v>
-      </c>
-      <c r="C197">
-        <v>12</v>
-      </c>
-      <c r="D197" t="s">
-        <v>20</v>
-      </c>
-      <c r="E197" s="3">
-        <v>47.487810048759798</v>
-      </c>
-    </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A198" t="s">
-        <v>18</v>
-      </c>
-      <c r="B198">
-        <v>20</v>
-      </c>
-      <c r="C198">
-        <v>14</v>
-      </c>
-      <c r="D198" t="s">
-        <v>19</v>
-      </c>
-      <c r="E198" s="3">
-        <v>9.0045298862004195</v>
-      </c>
-    </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A199" t="s">
-        <v>18</v>
-      </c>
-      <c r="B199">
-        <v>20</v>
-      </c>
-      <c r="C199">
-        <v>15</v>
-      </c>
-      <c r="D199" t="s">
-        <v>20</v>
-      </c>
-      <c r="E199" s="3">
-        <v>20.851735860167562</v>
-      </c>
-    </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A200" t="s">
-        <v>18</v>
-      </c>
-      <c r="B200">
-        <v>20</v>
-      </c>
-      <c r="C200">
-        <v>16</v>
-      </c>
-      <c r="D200" t="s">
-        <v>2</v>
-      </c>
-      <c r="E200" s="3">
-        <v>0.36572328813368588</v>
-      </c>
-    </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A201" t="s">
-        <v>18</v>
-      </c>
-      <c r="B201">
-        <v>20</v>
-      </c>
-      <c r="C201">
-        <v>17</v>
-      </c>
-      <c r="D201" t="s">
-        <v>2</v>
-      </c>
-      <c r="E201" s="3">
-        <v>0.61462814996926873</v>
-      </c>
-    </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A202" t="s">
-        <v>18</v>
-      </c>
-      <c r="B202">
-        <v>20</v>
-      </c>
-      <c r="C202">
-        <v>18</v>
-      </c>
-      <c r="D202" t="s">
-        <v>19</v>
-      </c>
-      <c r="E202" s="3">
-        <v>17.784426161389511</v>
-      </c>
-    </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A203" t="s">
-        <v>18</v>
-      </c>
-      <c r="B203">
-        <v>20</v>
-      </c>
-      <c r="C203">
-        <v>19</v>
-      </c>
-      <c r="D203" t="s">
-        <v>20</v>
-      </c>
-      <c r="E203" s="3">
-        <v>21.577227635336023</v>
-      </c>
-    </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A204" t="s">
-        <v>18</v>
-      </c>
-      <c r="B204">
-        <v>20</v>
-      </c>
-      <c r="C204">
-        <v>20</v>
-      </c>
-      <c r="D204" t="s">
-        <v>2</v>
-      </c>
-      <c r="E204" s="3">
-        <v>0.25822741227440965</v>
-      </c>
-    </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A205" t="s">
-        <v>18</v>
-      </c>
-      <c r="B205">
-        <v>20</v>
-      </c>
-      <c r="C205">
-        <v>21</v>
-      </c>
-      <c r="D205" t="s">
-        <v>2</v>
-      </c>
-      <c r="E205" s="3">
-        <v>0.77259850630955451</v>
-      </c>
-    </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A206" t="s">
-        <v>18</v>
-      </c>
-      <c r="B206">
-        <v>20</v>
-      </c>
-      <c r="C206">
-        <v>22</v>
-      </c>
-      <c r="D206" t="s">
-        <v>19</v>
-      </c>
-      <c r="E206" s="3">
-        <v>4.7538082515007467</v>
-      </c>
-    </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A207" t="s">
-        <v>18</v>
-      </c>
-      <c r="B207">
-        <v>20</v>
-      </c>
-      <c r="C207">
-        <v>23</v>
-      </c>
-      <c r="D207" t="s">
-        <v>19</v>
-      </c>
-      <c r="E207" s="3">
-        <v>5.8993923979087182</v>
-      </c>
-    </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A208" t="s">
-        <v>18</v>
-      </c>
-      <c r="B208">
-        <v>20</v>
-      </c>
-      <c r="C208">
-        <v>24</v>
-      </c>
-      <c r="D208" t="s">
-        <v>20</v>
-      </c>
-      <c r="E208" s="3">
-        <v>117.60964548420995</v>
-      </c>
-    </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A209" t="s">
-        <v>18</v>
-      </c>
-      <c r="B209">
-        <v>20</v>
-      </c>
-      <c r="C209">
-        <v>25</v>
-      </c>
-      <c r="D209" t="s">
-        <v>20</v>
-      </c>
-      <c r="E209" s="3">
-        <v>31.239992883828506</v>
-      </c>
-    </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A210" t="s">
-        <v>18</v>
-      </c>
-      <c r="B210">
-        <v>26</v>
-      </c>
-      <c r="C210">
-        <v>3</v>
-      </c>
-      <c r="D210" t="s">
-        <v>19</v>
-      </c>
-      <c r="E210" s="3">
-        <v>41.405342624854825</v>
-      </c>
-    </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A211" t="s">
-        <v>18</v>
-      </c>
-      <c r="B211">
-        <v>26</v>
-      </c>
-      <c r="C211">
-        <v>4</v>
-      </c>
-      <c r="D211" t="s">
-        <v>19</v>
-      </c>
-      <c r="E211" s="3">
-        <v>36.976274608783449</v>
-      </c>
-    </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A212" t="s">
-        <v>18</v>
-      </c>
-      <c r="B212">
-        <v>26</v>
-      </c>
-      <c r="C212">
-        <v>5</v>
-      </c>
-      <c r="D212" t="s">
-        <v>20</v>
-      </c>
-      <c r="E212" s="3">
-        <v>123.61755262219052</v>
-      </c>
-    </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A213" t="s">
-        <v>18</v>
-      </c>
-      <c r="B213">
-        <v>26</v>
-      </c>
-      <c r="C213">
-        <v>6</v>
-      </c>
-      <c r="D213" t="s">
-        <v>20</v>
-      </c>
-      <c r="E213" s="3">
-        <v>48.457411133467474</v>
-      </c>
-    </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A214" t="s">
-        <v>18</v>
-      </c>
-      <c r="B214">
-        <v>26</v>
-      </c>
-      <c r="C214">
-        <v>9</v>
-      </c>
-      <c r="D214" t="s">
-        <v>19</v>
-      </c>
-      <c r="E214" s="3">
-        <v>34.907260491327897</v>
-      </c>
-    </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A215" t="s">
-        <v>18</v>
-      </c>
-      <c r="B215">
-        <v>26</v>
-      </c>
-      <c r="C215">
-        <v>10</v>
-      </c>
-      <c r="D215" t="s">
-        <v>19</v>
-      </c>
-      <c r="E215" s="3">
-        <v>8.3572969086987783</v>
-      </c>
-    </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A216" t="s">
-        <v>18</v>
-      </c>
-      <c r="B216">
-        <v>26</v>
-      </c>
-      <c r="C216">
-        <v>11</v>
-      </c>
-      <c r="D216" t="s">
-        <v>20</v>
-      </c>
-      <c r="E216" s="3">
-        <v>50.16587915954559</v>
-      </c>
-    </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A217" t="s">
-        <v>18</v>
-      </c>
-      <c r="B217">
-        <v>26</v>
-      </c>
-      <c r="C217">
-        <v>12</v>
-      </c>
       <c r="D217" t="s">
         <v>20</v>
       </c>
       <c r="E217" s="3">
-        <v>26.253201609952434</v>
-      </c>
-    </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.2">
+        <v>3.1291789248462152</v>
+      </c>
+      <c r="F217">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B218">
-        <v>26</v>
+        <v>83</v>
       </c>
       <c r="C218">
         <v>14</v>
       </c>
       <c r="D218" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E218" s="3">
-        <v>1.019367991845056</v>
-      </c>
-    </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.2">
+        <v>1.1041902604756511</v>
+      </c>
+      <c r="F218">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="219" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
+        <v>21</v>
+      </c>
+      <c r="B219">
+        <v>83</v>
+      </c>
+      <c r="C219">
         <v>18</v>
       </c>
-      <c r="B219">
-        <v>26</v>
-      </c>
-      <c r="C219">
-        <v>15</v>
-      </c>
       <c r="D219" t="s">
         <v>20</v>
       </c>
       <c r="E219" s="3">
-        <v>100.01660485968894</v>
-      </c>
-    </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.2">
+        <v>1.371951219512195</v>
+      </c>
+      <c r="F219">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="220" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
+        <v>21</v>
+      </c>
+      <c r="B220">
+        <v>83</v>
+      </c>
+      <c r="C220">
+        <v>19</v>
+      </c>
+      <c r="D220" t="s">
+        <v>20</v>
+      </c>
+      <c r="E220" s="3">
+        <v>0.29062087186261559</v>
+      </c>
+      <c r="F220">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A221" t="s">
+        <v>21</v>
+      </c>
+      <c r="B221">
+        <v>83</v>
+      </c>
+      <c r="C221">
+        <v>23</v>
+      </c>
+      <c r="D221" t="s">
+        <v>20</v>
+      </c>
+      <c r="E221" s="3">
+        <v>5.0803945412782054</v>
+      </c>
+      <c r="F221">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A222" t="s">
+        <v>21</v>
+      </c>
+      <c r="B222">
+        <v>83</v>
+      </c>
+      <c r="C222">
+        <v>30</v>
+      </c>
+      <c r="D222" t="s">
+        <v>19</v>
+      </c>
+      <c r="E222" s="3">
+        <v>4.9995270717634819</v>
+      </c>
+      <c r="F222">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A223" t="s">
+        <v>21</v>
+      </c>
+      <c r="B223">
+        <v>83</v>
+      </c>
+      <c r="C223">
+        <v>31</v>
+      </c>
+      <c r="D223" t="s">
+        <v>19</v>
+      </c>
+      <c r="E223" s="3">
+        <v>0.11557520334012339</v>
+      </c>
+      <c r="F223">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="224" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A224" t="s">
+        <v>21</v>
+      </c>
+      <c r="B224">
+        <v>83</v>
+      </c>
+      <c r="C224">
+        <v>33</v>
+      </c>
+      <c r="D224" t="s">
+        <v>20</v>
+      </c>
+      <c r="E224" s="3">
+        <v>16.049739733950261</v>
+      </c>
+      <c r="F224">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A225" t="s">
+        <v>21</v>
+      </c>
+      <c r="B225">
+        <v>83</v>
+      </c>
+      <c r="C225">
+        <v>48</v>
+      </c>
+      <c r="D225" t="s">
+        <v>20</v>
+      </c>
+      <c r="E225" s="3">
+        <v>15.970909090909092</v>
+      </c>
+      <c r="F225">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="226" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A226" t="s">
+        <v>21</v>
+      </c>
+      <c r="B226">
+        <v>138</v>
+      </c>
+      <c r="C226">
+        <v>6</v>
+      </c>
+      <c r="D226" t="s">
+        <v>20</v>
+      </c>
+      <c r="E226" s="3">
+        <v>2.0163020163020162</v>
+      </c>
+      <c r="F226">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A227" t="s">
+        <v>21</v>
+      </c>
+      <c r="B227">
+        <v>138</v>
+      </c>
+      <c r="C227">
+        <v>11</v>
+      </c>
+      <c r="D227" t="s">
+        <v>20</v>
+      </c>
+      <c r="E227" s="3">
+        <v>0.67995492870186891</v>
+      </c>
+      <c r="F227">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A228" t="s">
+        <v>21</v>
+      </c>
+      <c r="B228">
+        <v>138</v>
+      </c>
+      <c r="C228">
         <v>18</v>
       </c>
-      <c r="B220">
-        <v>26</v>
-      </c>
-      <c r="C220">
-        <v>18</v>
-      </c>
-      <c r="D220" t="s">
-        <v>19</v>
-      </c>
-      <c r="E220" s="3">
-        <v>37.869210435582119</v>
-      </c>
-    </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A221" t="s">
-        <v>18</v>
-      </c>
-      <c r="B221">
-        <v>26</v>
-      </c>
-      <c r="C221">
-        <v>19</v>
-      </c>
-      <c r="D221" t="s">
-        <v>20</v>
-      </c>
-      <c r="E221" s="3">
-        <v>6.5579581708613972</v>
-      </c>
-    </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A222" t="s">
-        <v>18</v>
-      </c>
-      <c r="B222">
-        <v>26</v>
-      </c>
-      <c r="C222">
-        <v>22</v>
-      </c>
-      <c r="D222" t="s">
-        <v>19</v>
-      </c>
-      <c r="E222" s="3">
-        <v>4.2358522534733982</v>
-      </c>
-    </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A223" t="s">
-        <v>18</v>
-      </c>
-      <c r="B223">
-        <v>26</v>
-      </c>
-      <c r="C223">
-        <v>23</v>
-      </c>
-      <c r="D223" t="s">
-        <v>19</v>
-      </c>
-      <c r="E223" s="3">
-        <v>18.016297428062131</v>
-      </c>
-    </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A224" t="s">
-        <v>18</v>
-      </c>
-      <c r="B224">
-        <v>26</v>
-      </c>
-      <c r="C224">
-        <v>24</v>
-      </c>
-      <c r="D224" t="s">
-        <v>20</v>
-      </c>
-      <c r="E224" s="3">
-        <v>59.676044330775788</v>
-      </c>
-    </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A225" t="s">
-        <v>18</v>
-      </c>
-      <c r="B225">
-        <v>26</v>
-      </c>
-      <c r="C225">
-        <v>25</v>
-      </c>
-      <c r="D225" t="s">
-        <v>20</v>
-      </c>
-      <c r="E225" s="3">
-        <v>4.5304777594728165</v>
-      </c>
-    </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A226" t="s">
-        <v>21</v>
-      </c>
-      <c r="B226">
-        <v>21</v>
-      </c>
-      <c r="C226">
-        <v>2</v>
-      </c>
-      <c r="D226" t="s">
-        <v>2</v>
-      </c>
-      <c r="E226" s="3">
-        <v>0.2763957987838585</v>
-      </c>
-      <c r="F226">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A227" t="s">
-        <v>21</v>
-      </c>
-      <c r="B227">
-        <v>21</v>
-      </c>
-      <c r="C227">
-        <v>3</v>
-      </c>
-      <c r="D227" t="s">
-        <v>19</v>
-      </c>
-      <c r="E227" s="3">
-        <v>6.1667488899851994</v>
-      </c>
-      <c r="F227">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A228" t="s">
-        <v>21</v>
-      </c>
-      <c r="B228">
-        <v>21</v>
-      </c>
-      <c r="C228">
-        <v>4</v>
-      </c>
       <c r="D228" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="E228" s="3">
-        <v>0.18428424001179419</v>
+        <v>0.22289766970618033</v>
       </c>
       <c r="F228">
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>21</v>
       </c>
       <c r="B229">
-        <v>21</v>
+        <v>138</v>
       </c>
       <c r="C229">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="D229" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E229" s="3">
-        <v>6.6952914635033842</v>
+        <v>0.24703557312252963</v>
       </c>
       <c r="F229">
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>21</v>
       </c>
       <c r="B230">
-        <v>21</v>
+        <v>138</v>
       </c>
       <c r="C230">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D230" t="s">
         <v>20</v>
       </c>
+      <c r="E230" s="3">
+        <v>1.2177571128085907</v>
+      </c>
       <c r="F230">
-        <v>1</v>
-      </c>
-      <c r="G230" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>21</v>
       </c>
       <c r="B231">
-        <v>21</v>
+        <v>138</v>
       </c>
       <c r="C231">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="D231" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E231" s="3">
-        <v>0.74211502782931349</v>
+        <v>3.2207993791230112</v>
       </c>
       <c r="F231">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="232" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>21</v>
       </c>
       <c r="B232">
-        <v>21</v>
+        <v>138</v>
       </c>
       <c r="C232">
+        <v>33</v>
+      </c>
+      <c r="D232" t="s">
+        <v>20</v>
+      </c>
+      <c r="E232" s="3">
+        <v>17.403767403767404</v>
+      </c>
+      <c r="F232">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A233" t="s">
+        <v>21</v>
+      </c>
+      <c r="B233">
+        <v>138</v>
+      </c>
+      <c r="C233">
+        <v>48</v>
+      </c>
+      <c r="D233" t="s">
+        <v>20</v>
+      </c>
+      <c r="E233" s="3">
+        <v>2.4864144365836154</v>
+      </c>
+      <c r="F233">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="234" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A234" t="s">
+        <v>22</v>
+      </c>
+      <c r="B234">
+        <v>77</v>
+      </c>
+      <c r="C234">
         <v>9</v>
       </c>
-      <c r="D232" t="s">
-        <v>19</v>
-      </c>
-      <c r="E232" s="3">
-        <v>15.261446084563422</v>
-      </c>
-      <c r="F232">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A233" t="s">
-        <v>21</v>
-      </c>
-      <c r="B233">
-        <v>21</v>
-      </c>
-      <c r="C233">
-        <v>10</v>
-      </c>
-      <c r="D233" t="s">
-        <v>19</v>
-      </c>
-      <c r="F233">
-        <v>1</v>
-      </c>
-      <c r="G233" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A234" t="s">
-        <v>21</v>
-      </c>
-      <c r="B234">
-        <v>21</v>
-      </c>
-      <c r="C234">
+      <c r="D234" t="s">
+        <v>20</v>
+      </c>
+      <c r="E234" s="3">
+        <v>43.536039289325437</v>
+      </c>
+    </row>
+    <row r="235" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A235" t="s">
+        <v>22</v>
+      </c>
+      <c r="B235">
+        <v>77</v>
+      </c>
+      <c r="C235">
         <v>11</v>
       </c>
-      <c r="D234" t="s">
-        <v>20</v>
-      </c>
-      <c r="E234" s="3">
-        <v>104.56226880394576</v>
-      </c>
-      <c r="F234">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A235" t="s">
-        <v>21</v>
-      </c>
-      <c r="B235">
-        <v>21</v>
-      </c>
-      <c r="C235">
-        <v>12</v>
-      </c>
       <c r="D235" t="s">
         <v>20</v>
       </c>
+      <c r="E235" s="3">
+        <v>26.42159678345778</v>
+      </c>
       <c r="F235">
         <v>1</v>
       </c>
-      <c r="G235" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="236" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B236">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="C236">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D236" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="E236" s="3">
-        <v>1.0822510822510825</v>
+        <v>73.664122137404576</v>
       </c>
       <c r="F236">
         <v>1</v>
       </c>
     </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B237">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="C237">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D237" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E237" s="3">
-        <v>31.99327498392919</v>
+        <v>6.7308961330341823</v>
       </c>
       <c r="F237">
         <v>1</v>
       </c>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B238">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="C238">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D238" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E238" s="3">
-        <v>4.4904661371937928</v>
+        <v>27.935578330893119</v>
       </c>
       <c r="F238">
         <v>1</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B239">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="C239">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="D239" t="s">
         <v>19</v>
       </c>
       <c r="E239" s="3">
-        <v>10.916747651441529</v>
+        <v>7.896806669812805</v>
       </c>
       <c r="F239">
         <v>1</v>
       </c>
     </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B240">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="C240">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D240" t="s">
         <v>19</v>
       </c>
       <c r="E240" s="3">
-        <v>35.679978043090436</v>
+        <v>10.288722284255861</v>
       </c>
       <c r="F240">
         <v>1</v>
@@ -5382,19 +5502,19 @@
     </row>
     <row r="241" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B241">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="C241">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="D241" t="s">
         <v>20</v>
       </c>
       <c r="E241" s="3">
-        <v>198.10997218305835</v>
+        <v>14.649963154016211</v>
       </c>
       <c r="F241">
         <v>1</v>
@@ -5402,826 +5522,30 @@
     </row>
     <row r="242" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B242">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="C242">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="D242" t="s">
         <v>20</v>
       </c>
       <c r="E242" s="3">
-        <v>120.27829739752552</v>
+        <v>2.9397433815169727</v>
       </c>
       <c r="F242">
         <v>1</v>
       </c>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A243" t="s">
-        <v>21</v>
-      </c>
-      <c r="B243">
-        <v>21</v>
-      </c>
-      <c r="C243">
-        <v>20</v>
-      </c>
-      <c r="D243" t="s">
-        <v>2</v>
-      </c>
-      <c r="E243" s="3">
-        <v>0.42121634319411594</v>
-      </c>
-      <c r="F243">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A244" t="s">
-        <v>21</v>
-      </c>
-      <c r="B244">
-        <v>21</v>
-      </c>
-      <c r="C244">
-        <v>21</v>
-      </c>
-      <c r="D244" t="s">
-        <v>19</v>
-      </c>
-      <c r="E244" s="3">
-        <v>21.348717447280077</v>
-      </c>
-      <c r="F244">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A245" t="s">
-        <v>21</v>
-      </c>
-      <c r="B245">
-        <v>21</v>
-      </c>
-      <c r="C245">
-        <v>22</v>
-      </c>
-      <c r="D245" t="s">
-        <v>19</v>
-      </c>
-      <c r="E245" s="3">
-        <v>7.5543545019039424</v>
-      </c>
-      <c r="F245">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A246" t="s">
-        <v>21</v>
-      </c>
-      <c r="B246">
-        <v>21</v>
-      </c>
-      <c r="C246">
-        <v>23</v>
-      </c>
-      <c r="D246" t="s">
-        <v>20</v>
-      </c>
-      <c r="E246" s="3">
-        <v>98.704866562009414</v>
-      </c>
-      <c r="F246">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A247" t="s">
-        <v>21</v>
-      </c>
-      <c r="B247">
-        <v>21</v>
-      </c>
-      <c r="C247">
-        <v>30</v>
-      </c>
-      <c r="D247" t="s">
-        <v>19</v>
-      </c>
-      <c r="E247" s="3">
-        <v>15.60758082497213</v>
-      </c>
-      <c r="F247">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A248" t="s">
-        <v>21</v>
-      </c>
-      <c r="B248">
-        <v>21</v>
-      </c>
-      <c r="C248">
-        <v>31</v>
-      </c>
-      <c r="D248" t="s">
-        <v>19</v>
-      </c>
-      <c r="E248" s="3">
-        <v>50.821000810494404</v>
-      </c>
-      <c r="F248">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A249" t="s">
-        <v>21</v>
-      </c>
-      <c r="B249">
-        <v>21</v>
-      </c>
-      <c r="C249">
-        <v>32</v>
-      </c>
-      <c r="D249" t="s">
-        <v>20</v>
-      </c>
-      <c r="E249" s="3">
-        <v>78.636660143509459</v>
-      </c>
-      <c r="F249">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A250" t="s">
-        <v>21</v>
-      </c>
-      <c r="B250">
-        <v>21</v>
-      </c>
-      <c r="C250">
-        <v>33</v>
-      </c>
-      <c r="D250" t="s">
-        <v>20</v>
-      </c>
-      <c r="E250" s="3">
-        <v>143.13526324699509</v>
-      </c>
-      <c r="F250">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A251" t="s">
-        <v>21</v>
-      </c>
-      <c r="B251">
-        <v>21</v>
-      </c>
-      <c r="C251">
-        <v>34</v>
-      </c>
-      <c r="D251" t="s">
-        <v>20</v>
-      </c>
-      <c r="E251" s="3">
-        <v>53.602376825947019</v>
-      </c>
-      <c r="F251">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A252" t="s">
-        <v>21</v>
-      </c>
-      <c r="B252">
-        <v>21</v>
-      </c>
-      <c r="C252">
-        <v>45</v>
-      </c>
-      <c r="D252" t="s">
-        <v>19</v>
-      </c>
-      <c r="E252" s="3">
-        <v>11.229837337507655</v>
-      </c>
-      <c r="F252">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A253" t="s">
-        <v>21</v>
-      </c>
-      <c r="B253">
-        <v>21</v>
-      </c>
-      <c r="C253">
-        <v>46</v>
-      </c>
-      <c r="D253" t="s">
-        <v>19</v>
-      </c>
-      <c r="E253" s="3">
-        <v>23.619957537154985</v>
-      </c>
-      <c r="F253">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A254" t="s">
-        <v>21</v>
-      </c>
-      <c r="B254">
-        <v>21</v>
-      </c>
-      <c r="C254">
-        <v>47</v>
-      </c>
-      <c r="D254" t="s">
-        <v>20</v>
-      </c>
-      <c r="E254" s="3">
-        <v>95.876870940412317</v>
-      </c>
-      <c r="F254">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A255" t="s">
-        <v>21</v>
-      </c>
-      <c r="B255">
-        <v>21</v>
-      </c>
-      <c r="C255">
-        <v>48</v>
-      </c>
-      <c r="D255" t="s">
-        <v>20</v>
-      </c>
-      <c r="E255" s="3">
-        <v>195.71214629147946</v>
-      </c>
-      <c r="F255">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A256" t="s">
-        <v>21</v>
-      </c>
-      <c r="B256">
-        <v>83</v>
-      </c>
-      <c r="C256">
-        <v>6</v>
-      </c>
-      <c r="D256" t="s">
-        <v>20</v>
-      </c>
-      <c r="E256" s="3">
-        <v>3.0286786384347364</v>
-      </c>
-      <c r="F256">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A257" t="s">
-        <v>21</v>
-      </c>
-      <c r="B257">
-        <v>83</v>
-      </c>
-      <c r="C257">
-        <v>11</v>
-      </c>
-      <c r="D257" t="s">
-        <v>20</v>
-      </c>
-      <c r="E257" s="3">
-        <v>3.1291789248462152</v>
-      </c>
-      <c r="F257">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="258" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A258" t="s">
-        <v>21</v>
-      </c>
-      <c r="B258">
-        <v>83</v>
-      </c>
-      <c r="C258">
-        <v>14</v>
-      </c>
-      <c r="D258" t="s">
-        <v>20</v>
-      </c>
-      <c r="E258" s="3">
-        <v>1.1041902604756511</v>
-      </c>
-      <c r="F258">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A259" t="s">
-        <v>21</v>
-      </c>
-      <c r="B259">
-        <v>83</v>
-      </c>
-      <c r="C259">
-        <v>18</v>
-      </c>
-      <c r="D259" t="s">
-        <v>20</v>
-      </c>
-      <c r="E259" s="3">
-        <v>1.371951219512195</v>
-      </c>
-      <c r="F259">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A260" t="s">
-        <v>21</v>
-      </c>
-      <c r="B260">
-        <v>83</v>
-      </c>
-      <c r="C260">
-        <v>19</v>
-      </c>
-      <c r="D260" t="s">
-        <v>20</v>
-      </c>
-      <c r="E260" s="3">
-        <v>0.29062087186261559</v>
-      </c>
-      <c r="F260">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A261" t="s">
-        <v>21</v>
-      </c>
-      <c r="B261">
-        <v>83</v>
-      </c>
-      <c r="C261">
-        <v>23</v>
-      </c>
-      <c r="D261" t="s">
-        <v>20</v>
-      </c>
-      <c r="E261" s="3">
-        <v>5.0803945412782054</v>
-      </c>
-      <c r="F261">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A262" t="s">
-        <v>21</v>
-      </c>
-      <c r="B262">
-        <v>83</v>
-      </c>
-      <c r="C262">
-        <v>30</v>
-      </c>
-      <c r="D262" t="s">
-        <v>19</v>
-      </c>
-      <c r="E262" s="3">
-        <v>4.9995270717634819</v>
-      </c>
-      <c r="F262">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A263" t="s">
-        <v>21</v>
-      </c>
-      <c r="B263">
-        <v>83</v>
-      </c>
-      <c r="C263">
-        <v>31</v>
-      </c>
-      <c r="D263" t="s">
-        <v>19</v>
-      </c>
-      <c r="E263" s="3">
-        <v>0.11557520334012339</v>
-      </c>
-      <c r="F263">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A264" t="s">
-        <v>21</v>
-      </c>
-      <c r="B264">
-        <v>83</v>
-      </c>
-      <c r="C264">
-        <v>33</v>
-      </c>
-      <c r="D264" t="s">
-        <v>20</v>
-      </c>
-      <c r="E264" s="3">
-        <v>16.049739733950261</v>
-      </c>
-      <c r="F264">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A265" t="s">
-        <v>21</v>
-      </c>
-      <c r="B265">
-        <v>83</v>
-      </c>
-      <c r="C265">
-        <v>48</v>
-      </c>
-      <c r="D265" t="s">
-        <v>20</v>
-      </c>
-      <c r="E265" s="3">
-        <v>15.970909090909092</v>
-      </c>
-      <c r="F265">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A266" t="s">
-        <v>21</v>
-      </c>
-      <c r="B266">
-        <v>138</v>
-      </c>
-      <c r="C266">
-        <v>6</v>
-      </c>
-      <c r="D266" t="s">
-        <v>20</v>
-      </c>
-      <c r="E266" s="3">
-        <v>2.0163020163020162</v>
-      </c>
-      <c r="F266">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A267" t="s">
-        <v>21</v>
-      </c>
-      <c r="B267">
-        <v>138</v>
-      </c>
-      <c r="C267">
-        <v>11</v>
-      </c>
-      <c r="D267" t="s">
-        <v>20</v>
-      </c>
-      <c r="E267" s="3">
-        <v>0.67995492870186891</v>
-      </c>
-      <c r="F267">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A268" t="s">
-        <v>21</v>
-      </c>
-      <c r="B268">
-        <v>138</v>
-      </c>
-      <c r="C268">
-        <v>18</v>
-      </c>
-      <c r="D268" t="s">
-        <v>20</v>
-      </c>
-      <c r="E268" s="3">
-        <v>0.22289766970618033</v>
-      </c>
-      <c r="F268">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A269" t="s">
-        <v>21</v>
-      </c>
-      <c r="B269">
-        <v>138</v>
-      </c>
-      <c r="C269">
-        <v>19</v>
-      </c>
-      <c r="D269" t="s">
-        <v>20</v>
-      </c>
-      <c r="E269" s="3">
-        <v>0.24703557312252963</v>
-      </c>
-      <c r="F269">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A270" t="s">
-        <v>21</v>
-      </c>
-      <c r="B270">
-        <v>138</v>
-      </c>
-      <c r="C270">
-        <v>23</v>
-      </c>
-      <c r="D270" t="s">
-        <v>20</v>
-      </c>
-      <c r="E270" s="3">
-        <v>1.2177571128085907</v>
-      </c>
-      <c r="F270">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A271" t="s">
-        <v>21</v>
-      </c>
-      <c r="B271">
-        <v>138</v>
-      </c>
-      <c r="C271">
-        <v>30</v>
-      </c>
-      <c r="D271" t="s">
-        <v>19</v>
-      </c>
-      <c r="E271" s="3">
-        <v>3.2207993791230112</v>
-      </c>
-      <c r="F271">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="272" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A272" t="s">
-        <v>21</v>
-      </c>
-      <c r="B272">
-        <v>138</v>
-      </c>
-      <c r="C272">
-        <v>33</v>
-      </c>
-      <c r="D272" t="s">
-        <v>20</v>
-      </c>
-      <c r="E272" s="3">
-        <v>17.403767403767404</v>
-      </c>
-      <c r="F272">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="273" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A273" t="s">
-        <v>21</v>
-      </c>
-      <c r="B273">
-        <v>138</v>
-      </c>
-      <c r="C273">
-        <v>48</v>
-      </c>
-      <c r="D273" t="s">
-        <v>20</v>
-      </c>
-      <c r="E273" s="3">
-        <v>2.4864144365836154</v>
-      </c>
-      <c r="F273">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="274" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A274" t="s">
-        <v>22</v>
-      </c>
-      <c r="B274">
-        <v>77</v>
-      </c>
-      <c r="C274">
-        <v>9</v>
-      </c>
-      <c r="D274" t="s">
-        <v>20</v>
-      </c>
-      <c r="E274" s="3">
-        <v>43.536039289325437</v>
-      </c>
-    </row>
-    <row r="275" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A275" t="s">
-        <v>22</v>
-      </c>
-      <c r="B275">
-        <v>77</v>
-      </c>
-      <c r="C275">
-        <v>11</v>
-      </c>
-      <c r="D275" t="s">
-        <v>20</v>
-      </c>
-      <c r="E275" s="3">
-        <v>26.42159678345778</v>
-      </c>
-      <c r="F275">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="276" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A276" t="s">
-        <v>22</v>
-      </c>
-      <c r="B276">
-        <v>77</v>
-      </c>
-      <c r="C276">
-        <v>16</v>
-      </c>
-      <c r="D276" t="s">
-        <v>20</v>
-      </c>
-      <c r="E276" s="3">
-        <v>73.664122137404576</v>
-      </c>
-      <c r="F276">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="277" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A277" t="s">
-        <v>22</v>
-      </c>
-      <c r="B277">
-        <v>77</v>
-      </c>
-      <c r="C277">
-        <v>19</v>
-      </c>
-      <c r="D277" t="s">
-        <v>19</v>
-      </c>
-      <c r="E277" s="3">
-        <v>6.7308961330341823</v>
-      </c>
-      <c r="F277">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="278" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A278" t="s">
-        <v>22</v>
-      </c>
-      <c r="B278">
-        <v>77</v>
-      </c>
-      <c r="C278">
-        <v>24</v>
-      </c>
-      <c r="D278" t="s">
-        <v>19</v>
-      </c>
-      <c r="E278" s="3">
-        <v>27.935578330893119</v>
-      </c>
-      <c r="F278">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A279" t="s">
-        <v>22</v>
-      </c>
-      <c r="B279">
-        <v>77</v>
-      </c>
-      <c r="C279">
-        <v>30</v>
-      </c>
-      <c r="D279" t="s">
-        <v>19</v>
-      </c>
-      <c r="E279" s="3">
-        <v>7.896806669812805</v>
-      </c>
-      <c r="F279">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="280" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A280" t="s">
-        <v>22</v>
-      </c>
-      <c r="B280">
-        <v>77</v>
-      </c>
-      <c r="C280">
-        <v>31</v>
-      </c>
-      <c r="D280" t="s">
-        <v>19</v>
-      </c>
-      <c r="E280" s="3">
-        <v>10.288722284255861</v>
-      </c>
-      <c r="F280">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="281" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A281" t="s">
-        <v>22</v>
-      </c>
-      <c r="B281">
-        <v>77</v>
-      </c>
-      <c r="C281">
-        <v>32</v>
-      </c>
-      <c r="D281" t="s">
-        <v>20</v>
-      </c>
-      <c r="E281" s="3">
-        <v>14.649963154016211</v>
-      </c>
-      <c r="F281">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="282" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A282" t="s">
-        <v>22</v>
-      </c>
-      <c r="B282">
-        <v>77</v>
-      </c>
-      <c r="C282">
-        <v>37</v>
-      </c>
-      <c r="D282" t="s">
-        <v>20</v>
-      </c>
-      <c r="E282" s="3">
-        <v>2.9397433815169727</v>
-      </c>
-      <c r="F282">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G273">
-    <sortCondition ref="A2:A273"/>
-    <sortCondition ref="B2:B273"/>
-    <sortCondition ref="C2:C273"/>
+  <autoFilter ref="A1:G242" xr:uid="{28924032-712C-42DD-811A-811BE3665EE3}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G233">
+    <sortCondition ref="A2:A233"/>
+    <sortCondition ref="B2:B233"/>
+    <sortCondition ref="C2:C233"/>
   </sortState>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>